<commit_message>
Hojas de encargo de Drive: 2023; el adelanto de Next Generation va a la forma de pago
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cruce_hojas_2024.xlsx
+++ b/docs/cruce_hojas_2024.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -94,9 +89,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2178,14 +2170,14 @@
           <t>Y24_020a</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: PARA TI (Next Generation): adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 8.550 de 17.690 (proyecto 15.200 + LEE/IEE 2.490).</t>
+          <t>RESUELTO LEYENDO: Next Generation: adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 8.550 de 17.690 (proyecto 15.200 + LEE/IEE 2.490). (Mónica: el importe es el total de la hoja; la condición va en la forma de pago.)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2227,10 +2219,12 @@
 TRAMITACION LICENCIAS: sin precio propio</t>
         </is>
       </c>
-      <c r="K22" s="2" t="n"/>
+      <c r="K22" s="2" t="n">
+        <v>17690</v>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Adelanto 8.550 + IVA: un tercio a la firma, un tercio a la entrega del proyecto y un tercio a la dirección de obra; resto a la comunicación de la concesión de la subvención del Programa 5</t>
+          <t>Adelanto a cuenta 8.550 € + IVA a la firma; el resto. solo si se concede el programa 5.</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2846,14 +2840,14 @@
           <t>Y24_027</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: PARA TI (Next Generation): adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 8.500 de 28.050; si no se concede, los honorarios son el adelanto.</t>
+          <t>RESUELTO LEYENDO: Next Generation: adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 8.500 de 28.050; si no se concede, los honorarios son el adelanto. (Mónica: el importe es el total de la hoja; la condición va en la forma de pago.)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2900,7 +2894,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Adelanto (8.500 € + IVA): 50% al encargo + 50% a la entrega de proyecto. Resto: a la comunicación de la concesión de la subvención del Programa 5</t>
+          <t>Adelanto a cuenta 8.500 € + IVA a la firma; el resto. solo si se concede el programa 5.</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -5057,14 +5051,14 @@
           <t>Y24_052</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: PARA TI (Next Generation): adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Firma DIDEPRO (no la comunidad): adelanto 8.500; lo concedido menos 8.500 se reparte al 50% entre Accesalia y DIDEPRO. Firmada 'EN PAUSA'.</t>
+          <t>RESUELTO LEYENDO: Next Generation: adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Firma DIDEPRO (no la comunidad): adelanto 8.500; lo concedido menos 8.500 se reparte al 50% entre Accesalia y DIDEPRO. Firmada 'EN PAUSA'. (Mónica: el importe es el total de la hoja; la condición va en la forma de pago.)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -5109,7 +5103,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>50% al encargo y 50% a la entrega de proyecto</t>
+          <t>Adelanto a cuenta 8.500 € + IVA a la firma; el resto. solo si se concede el programa 5.</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
@@ -5943,14 +5937,14 @@
           <t>Y24_061</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: PARA TI (Next Generation): adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 5.500 de 11.370; tres hojas en el documento (proyecto, subvención, cesión de CAES).</t>
+          <t>RESUELTO LEYENDO: Next Generation: adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 5.500 de 11.370; tres hojas en el documento (proyecto, subvención, cesión de CAES). (Mónica: el importe es el total de la hoja; la condición va en la forma de pago.)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5994,11 +5988,11 @@
         </is>
       </c>
       <c r="K66" s="2" t="n">
-        <v>13350</v>
+        <v>11370</v>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Adelanto (5.500 € + IVA): 50% al encargo + 50% a la entrega de proyecto. Resto: a la comunicación de la concesión de la subvención del Programa 5</t>
+          <t>Adelanto a cuenta 5.500 € + IVA a la firma; el resto. solo si se concede el programa 5.</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
@@ -6042,14 +6036,14 @@
           <t>Y24_062</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: PARA TI (Next Generation): adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 7.220 de 16.110; dos hojas en el documento (proyecto y subvención).</t>
+          <t>RESUELTO LEYENDO: Next Generation: adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Adelanto 7.220 de 16.110; dos hojas en el documento (proyecto y subvención). (Mónica: el importe es el total de la hoja; la condición va en la forma de pago.)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -6092,11 +6086,11 @@
         </is>
       </c>
       <c r="K67" s="2" t="n">
-        <v>18090</v>
+        <v>16110</v>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Adelanto (7.220 € + IVA): 50% al encargo + 50% a la entrega de proyecto. Resto: a la comunicación de la concesión de la subvención del Programa 5</t>
+          <t>Adelanto a cuenta 7.220 € + IVA a la firma; el resto. solo si se concede el programa 5.</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
@@ -10873,14 +10867,14 @@
           <t>Y24_117</t>
         </is>
       </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: PARA TI (Next Generation): adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Firmada la de PROYECTO (SATE) del 21-05: adelanto 7.220 de 16.900.</t>
+          <t>RESUELTO LEYENDO: Next Generation: adelanto a cuenta + importe total que solo se cobra si se concede el programa 5. Firmada la de PROYECTO (SATE) del 21-05: adelanto 7.220 de 16.900. (Mónica: el importe es el total de la hoja; la condición va en la forma de pago.)</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -10923,10 +10917,12 @@
 TRAMITACION SUBVENCIONES: 1980 €</t>
         </is>
       </c>
-      <c r="K124" s="2" t="n"/>
+      <c r="K124" s="2" t="n">
+        <v>16900</v>
+      </c>
       <c r="L124" s="2" t="inlineStr">
         <is>
-          <t>Adelanto 7.220 + IVA: 50% al encargo + 50% a la entrega de proyecto; resto a la comunicación de la concesión de la subvención del Programa 5</t>
+          <t>Adelanto a cuenta 7.220 € + IVA a la firma; el resto. solo si se concede el programa 5.</t>
         </is>
       </c>
       <c r="M124" s="2" t="inlineStr">

</xml_diff>